<commit_message>
chore: update tweet data 2026-05-10T11:58:13Z
</commit_message>
<xml_diff>
--- a/data/milei_tweets.xlsx
+++ b/data/milei_tweets.xlsx
@@ -13269,7 +13269,7 @@
       </c>
       <c r="C571" t="inlineStr">
         <is>
-          <t>RT @altashanta: "En Estados Unidos está el presidente y calificaron su viaje como algo menor para no conseguir nada para Argentina… Consigu…</t>
+          <t>RT @DiegoMac227: 🇦🇷🇺🇸l Hoy les traigo un montón de hechos de que la libertad funciona. El primer mito que rompimos cuando llegamos a la adm…</t>
         </is>
       </c>
       <c r="D571" t="inlineStr">
@@ -13291,7 +13291,7 @@
       </c>
       <c r="C572" t="inlineStr">
         <is>
-          <t>RT @DiegoMac227: 🇦🇷🇺🇸l Hoy les traigo un montón de hechos de que la libertad funciona. El primer mito que rompimos cuando llegamos a la adm…</t>
+          <t>RT @altashanta: "En Estados Unidos está el presidente y calificaron su viaje como algo menor para no conseguir nada para Argentina… Consigu…</t>
         </is>
       </c>
       <c r="D572" t="inlineStr">

</xml_diff>